<commit_message>
Fix XML element order bug (cols/sheetFormatPr) that made the xlsx unreadable
Co-authored-by: valiyevtwo-eng <300492679+valiyevtwo-eng@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/IELTS_6_Oylik_Reja.xlsx
+++ b/IELTS_6_Oylik_Reja.xlsx
@@ -227,6 +227,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1:F57"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
     <col min="2" max="2" width="32" customWidth="1"/>
@@ -235,7 +236,6 @@
     <col min="5" max="5" width="32" customWidth="1"/>
     <col min="6" max="6" width="24" customWidth="1"/>
   </cols>
-  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -1710,6 +1710,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1:F203"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
     <col min="2" max="2" width="26" customWidth="1"/>
@@ -1718,7 +1719,6 @@
     <col min="5" max="5" width="30" customWidth="1"/>
     <col min="6" max="6" width="40" customWidth="1"/>
   </cols>
-  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -7995,6 +7995,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1:F203"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
     <col min="2" max="2" width="26" customWidth="1"/>
@@ -8003,7 +8004,6 @@
     <col min="5" max="5" width="30" customWidth="1"/>
     <col min="6" max="6" width="40" customWidth="1"/>
   </cols>
-  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -14280,6 +14280,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1:F203"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
     <col min="2" max="2" width="26" customWidth="1"/>
@@ -14288,7 +14289,6 @@
     <col min="5" max="5" width="30" customWidth="1"/>
     <col min="6" max="6" width="40" customWidth="1"/>
   </cols>
-  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -16225,7 +16225,7 @@
       </c>
       <c r="F68" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lug'at almashtirish - takrorlanган so'zlarni sinonim bilan almashtiring</t>
+          <t xml:space="preserve">Lug'at almashtirish - takrorlangan so'zlarni sinonim bilan almashtiring</t>
         </is>
       </c>
     </row>
@@ -16449,7 +16449,7 @@
       </c>
       <c r="F75" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lug'at almashtirish - takrorlanган so'zlarni sinonim bilan almashtiring</t>
+          <t xml:space="preserve">Lug'at almashtirish - takrorlangan so'zlarni sinonim bilan almashtiring</t>
         </is>
       </c>
     </row>
@@ -16673,7 +16673,7 @@
       </c>
       <c r="F82" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lug'at almashtirish - takrorlanган so'zlarni sinonim bilan almashtiring</t>
+          <t xml:space="preserve">Lug'at almashtirish - takrorlangan so'zlarni sinonim bilan almashtiring</t>
         </is>
       </c>
     </row>
@@ -16897,7 +16897,7 @@
       </c>
       <c r="F89" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lug'at almashtirish - takrorlanган so'zlarni sinonim bilan almashtiring</t>
+          <t xml:space="preserve">Lug'at almashtirish - takrorlangan so'zlarni sinonim bilan almashtiring</t>
         </is>
       </c>
     </row>
@@ -20565,6 +20565,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1:F212"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
     <col min="2" max="2" width="26" customWidth="1"/>
@@ -20573,7 +20574,6 @@
     <col min="5" max="5" width="32" customWidth="1"/>
     <col min="6" max="6" width="42" customWidth="1"/>
   </cols>
-  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">

</xml_diff>